<commit_message>
- Changes on get_* functions - Added a new executable file for the X13AS ASCII tool. - More
</commit_message>
<xml_diff>
--- a/src/pib_nowcast/data/last_data_at_time.xlsx
+++ b/src/pib_nowcast/data/last_data_at_time.xlsx
@@ -28101,45 +28101,21 @@
       <c r="K366" t="inlineStr"/>
       <c r="L366" t="inlineStr"/>
       <c r="M366" t="inlineStr"/>
-      <c r="N366" t="n">
-        <v>120.55</v>
-      </c>
-      <c r="O366" t="n">
-        <v>112.44</v>
-      </c>
-      <c r="P366" t="n">
-        <v>125.96</v>
-      </c>
-      <c r="Q366" t="n">
-        <v>88.7</v>
-      </c>
-      <c r="R366" t="n">
-        <v>91.7</v>
-      </c>
-      <c r="S366" t="n">
-        <v>85.8</v>
-      </c>
+      <c r="N366" t="inlineStr"/>
+      <c r="O366" t="inlineStr"/>
+      <c r="P366" t="inlineStr"/>
+      <c r="Q366" t="inlineStr"/>
+      <c r="R366" t="inlineStr"/>
+      <c r="S366" t="inlineStr"/>
       <c r="T366" t="inlineStr"/>
       <c r="U366" t="inlineStr"/>
       <c r="V366" t="inlineStr"/>
-      <c r="W366" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="X366" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="Y366" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="Z366" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="AA366" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="AB366" t="n">
-        <v>0.91</v>
-      </c>
+      <c r="W366" t="inlineStr"/>
+      <c r="X366" t="inlineStr"/>
+      <c r="Y366" t="inlineStr"/>
+      <c r="Z366" t="inlineStr"/>
+      <c r="AA366" t="inlineStr"/>
+      <c r="AB366" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -57935,45 +57911,21 @@
       <c r="K366" t="inlineStr"/>
       <c r="L366" t="inlineStr"/>
       <c r="M366" t="inlineStr"/>
-      <c r="N366" t="n">
-        <v>120.55</v>
-      </c>
-      <c r="O366" t="n">
-        <v>112.44</v>
-      </c>
-      <c r="P366" t="n">
-        <v>125.96</v>
-      </c>
-      <c r="Q366" t="n">
-        <v>88.7</v>
-      </c>
-      <c r="R366" t="n">
-        <v>91.7</v>
-      </c>
-      <c r="S366" t="n">
-        <v>85.8</v>
-      </c>
+      <c r="N366" t="inlineStr"/>
+      <c r="O366" t="inlineStr"/>
+      <c r="P366" t="inlineStr"/>
+      <c r="Q366" t="inlineStr"/>
+      <c r="R366" t="inlineStr"/>
+      <c r="S366" t="inlineStr"/>
       <c r="T366" t="inlineStr"/>
       <c r="U366" t="inlineStr"/>
       <c r="V366" t="inlineStr"/>
-      <c r="W366" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="X366" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="Y366" t="n">
-        <v>0.84</v>
-      </c>
-      <c r="Z366" t="n">
-        <v>0.87</v>
-      </c>
-      <c r="AA366" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="AB366" t="n">
-        <v>0.91</v>
-      </c>
+      <c r="W366" t="inlineStr"/>
+      <c r="X366" t="inlineStr"/>
+      <c r="Y366" t="inlineStr"/>
+      <c r="Z366" t="inlineStr"/>
+      <c r="AA366" t="inlineStr"/>
+      <c r="AB366" t="inlineStr"/>
       <c r="AC366" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>